<commit_message>
HU-042: columna de dependencia del aval de arquitectura en las tareas
Cada tarea marca si puede iniciar ya (nativo/declarativo/contratos), si es
parcial (la base avanza, la UI espera) o si espera el aval de Salesforce
sobre LWC vs OmniStudio.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARnTRs7x9qahUXJKvUM6vN
</commit_message>
<xml_diff>
--- a/deploy/hu042-seleccion-vehiculo/HU042_Guia_Tecnica.xlsx
+++ b/deploy/hu042-seleccion-vehiculo/HU042_Guia_Tecnica.xlsx
@@ -376,9 +376,10 @@
   </sheetPr>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="36" customWidth="1"/>
-    <col min="3" max="3" width="72" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="62" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -412,6 +413,11 @@
           <t xml:space="preserve">Componente de la guía</t>
         </is>
       </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">¿Espera el aval de Salesforce (LWC vs OmniStudio)?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -434,6 +440,11 @@
           <t xml:space="preserve">QuoteOrderService</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No — puede iniciar ya (nativo: Record Types, layouts y plantillas)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -456,6 +467,11 @@
           <t xml:space="preserve">ventaGuiadaAction</t>
         </is>
       </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí — es el componente de UI; la definición funcional de la acción no cambia</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -478,6 +494,11 @@
           <t xml:space="preserve">ventaVehiculo</t>
         </is>
       </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial — la lógica de búsqueda y filtros es neutral; la pantalla espera el aval</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -500,6 +521,11 @@
           <t xml:space="preserve">ventaUsados</t>
         </is>
       </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial — igual que la 3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -522,6 +548,11 @@
           <t xml:space="preserve">SapInventoryService</t>
         </is>
       </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial — el contrato del servicio MuleSoft puede avanzar ya; el mecanismo de invocación (Continuation o Integration Procedure) espera el aval</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -544,6 +575,11 @@
           <t xml:space="preserve">PricingService + QuoteOrderService</t>
         </is>
       </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No — BRE y Quote son nativos; la invocación se adapta al mecanismo aprobado</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -566,6 +602,11 @@
           <t xml:space="preserve">ventaVehiculo / ventaUsados</t>
         </is>
       </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial — Field History y Quotes por Oportunidad pueden configurarse ya; la UI espera</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -588,6 +629,11 @@
           <t xml:space="preserve">Flow declarativo</t>
         </is>
       </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No — Flow declarativo, puede iniciar ya</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -610,6 +656,11 @@
           <t xml:space="preserve">ventaVehiculo (variante)</t>
         </is>
       </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sí — variante de UI</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -630,6 +681,11 @@
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Todos</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parcial — los casos de prueba se escriben ya; la automatización sigue al mecanismo</t>
         </is>
       </c>
     </row>

</xml_diff>